<commit_message>
Update EMOData dashboard data
</commit_message>
<xml_diff>
--- a/public/exports-60-250-with-coowners/11259979.xlsx
+++ b/public/exports-60-250-with-coowners/11259979.xlsx
@@ -1466,30 +1466,30 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Segelckesvej 7</t>
+          <t xml:space="preserve">Niels Ebbesens Vej 21</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t xml:space="preserve">2000</t>
+          <t xml:space="preserve">1911</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t xml:space="preserve">100030239</t>
+          <t xml:space="preserve">100027029</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t xml:space="preserve">2</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="J20">
-        <v>197</v>
+        <v>190</v>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t xml:space="preserve">311223800</t>
+          <t xml:space="preserve">311230611</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
@@ -1499,7 +1499,7 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t xml:space="preserve">2027-01-21</t>
+          <t xml:space="preserve">2027-02-24</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
@@ -1541,30 +1541,30 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Niels Ebbesens Vej 21</t>
+          <t xml:space="preserve">Dronning Olgas Vej 6</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t xml:space="preserve">1911</t>
+          <t xml:space="preserve">2000</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t xml:space="preserve">100027029</t>
+          <t xml:space="preserve">100028120</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">2</t>
         </is>
       </c>
       <c r="J21">
-        <v>190</v>
+        <v>72</v>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t xml:space="preserve">311230611</t>
+          <t xml:space="preserve">311230652</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
@@ -1574,7 +1574,7 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t xml:space="preserve">2027-02-24</t>
+          <t xml:space="preserve">2027-02-25</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -1616,7 +1616,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dronning Olgas Vej 6</t>
+          <t xml:space="preserve">La Cours Vej 2A</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1626,7 +1626,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t xml:space="preserve">100028120</t>
+          <t xml:space="preserve">100030249</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1635,11 +1635,11 @@
         </is>
       </c>
       <c r="J22">
-        <v>72</v>
+        <v>150</v>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t xml:space="preserve">311230652</t>
+          <t xml:space="preserve">311231520</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
@@ -1649,7 +1649,7 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t xml:space="preserve">2027-02-25</t>
+          <t xml:space="preserve">2027-03-01</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
@@ -1686,35 +1686,35 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t xml:space="preserve">147</t>
+          <t xml:space="preserve">306</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t xml:space="preserve">La Cours Vej 2A</t>
+          <t xml:space="preserve">Skærbygårdsvej 15</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t xml:space="preserve">2000</t>
+          <t xml:space="preserve">4500</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t xml:space="preserve">100030249</t>
+          <t xml:space="preserve">5347084</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t xml:space="preserve">2</t>
+          <t xml:space="preserve">3</t>
         </is>
       </c>
       <c r="J23">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t xml:space="preserve">311231520</t>
+          <t xml:space="preserve">311231683</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
@@ -1724,7 +1724,7 @@
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t xml:space="preserve">2027-03-01</t>
+          <t xml:space="preserve">2027-03-02</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
@@ -1761,35 +1761,35 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t xml:space="preserve">306</t>
+          <t xml:space="preserve">147</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Skærbygårdsvej 15</t>
+          <t xml:space="preserve">Skellet 27A</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t xml:space="preserve">4500</t>
+          <t xml:space="preserve">2000</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t xml:space="preserve">5347084</t>
+          <t xml:space="preserve">100029530</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t xml:space="preserve">3</t>
+          <t xml:space="preserve">5</t>
         </is>
       </c>
       <c r="J24">
-        <v>144</v>
+        <v>224</v>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t xml:space="preserve">311231683</t>
+          <t xml:space="preserve">311233769</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
@@ -1799,7 +1799,7 @@
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t xml:space="preserve">2027-03-02</t>
+          <t xml:space="preserve">2027-03-13</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
@@ -1841,30 +1841,30 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Skellet 27A</t>
+          <t xml:space="preserve">Vodroffsvej 44</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t xml:space="preserve">2000</t>
+          <t xml:space="preserve">1900</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t xml:space="preserve">100029530</t>
+          <t xml:space="preserve">100027252</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t xml:space="preserve">5</t>
+          <t xml:space="preserve">2</t>
         </is>
       </c>
       <c r="J25">
-        <v>224</v>
+        <v>178</v>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t xml:space="preserve">311233769</t>
+          <t xml:space="preserve">311234441</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
@@ -1874,7 +1874,7 @@
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t xml:space="preserve">2027-03-13</t>
+          <t xml:space="preserve">2027-03-15</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
@@ -1916,30 +1916,30 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vodroffsvej 44</t>
+          <t xml:space="preserve">Edisonsvej 3</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t xml:space="preserve">1900</t>
+          <t xml:space="preserve">1856</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t xml:space="preserve">100027252</t>
+          <t xml:space="preserve">100025577</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t xml:space="preserve">2</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="J26">
-        <v>178</v>
+        <v>228</v>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t xml:space="preserve">311234441</t>
+          <t xml:space="preserve">311247695</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
@@ -1949,7 +1949,7 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t xml:space="preserve">2027-03-15</t>
+          <t xml:space="preserve">2027-05-16</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
@@ -1991,40 +1991,40 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Edisonsvej 3</t>
+          <t xml:space="preserve">Nyelandsvej 70</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t xml:space="preserve">1856</t>
+          <t xml:space="preserve">2000</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t xml:space="preserve">100025577</t>
+          <t xml:space="preserve">100029712</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">2</t>
         </is>
       </c>
       <c r="J27">
-        <v>228</v>
+        <v>126</v>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t xml:space="preserve">311247695</t>
+          <t xml:space="preserve">311379735</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Energitjenesten Øst</t>
+          <t xml:space="preserve">Topdahl Energirådgivere ApS</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t xml:space="preserve">2027-05-16</t>
+          <t xml:space="preserve">2029-05-29</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
@@ -2066,7 +2066,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nyelandsvej 70</t>
+          <t xml:space="preserve">Hoffmeyersvej 32</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -2076,30 +2076,30 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t xml:space="preserve">100029712</t>
+          <t xml:space="preserve">100029488</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t xml:space="preserve">2</t>
+          <t xml:space="preserve">3</t>
         </is>
       </c>
       <c r="J28">
-        <v>126</v>
+        <v>111</v>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t xml:space="preserve">311379735</t>
+          <t xml:space="preserve">311718500</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Topdahl Energirådgivere ApS</t>
+          <t xml:space="preserve">OBH Ingeniørservice A/S</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t xml:space="preserve">2029-05-29</t>
+          <t xml:space="preserve">2033-10-30</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
@@ -2141,7 +2141,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hoffmeyersvej 32</t>
+          <t xml:space="preserve">Nyelandsvej 23A</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -2151,7 +2151,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t xml:space="preserve">100029488</t>
+          <t xml:space="preserve">100025833</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -2160,11 +2160,11 @@
         </is>
       </c>
       <c r="J29">
-        <v>111</v>
+        <v>237</v>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t xml:space="preserve">311718500</t>
+          <t xml:space="preserve">311722647</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
@@ -2174,7 +2174,7 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t xml:space="preserve">2033-10-30</t>
+          <t xml:space="preserve">2033-11-16</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
@@ -2216,30 +2216,30 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nyelandsvej 23A</t>
+          <t xml:space="preserve">Frederiksberg Alle 63</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t xml:space="preserve">2000</t>
+          <t xml:space="preserve">1820</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t xml:space="preserve">100025833</t>
+          <t xml:space="preserve">100028276</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t xml:space="preserve">3</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="J30">
-        <v>237</v>
+        <v>130</v>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t xml:space="preserve">311722647</t>
+          <t xml:space="preserve">311723249</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
@@ -2249,7 +2249,7 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t xml:space="preserve">2033-11-16</t>
+          <t xml:space="preserve">2033-11-19</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
@@ -2306,15 +2306,15 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">4</t>
         </is>
       </c>
       <c r="J31">
-        <v>130</v>
+        <v>146</v>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t xml:space="preserve">311723249</t>
+          <t xml:space="preserve">311734449</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
@@ -2324,7 +2324,7 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t xml:space="preserve">2033-11-19</t>
+          <t xml:space="preserve">2034-01-22</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
@@ -2366,30 +2366,30 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Frederiksberg Alle 63</t>
+          <t xml:space="preserve">Godthåbsvej 21C</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t xml:space="preserve">1820</t>
+          <t xml:space="preserve">2000</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t xml:space="preserve">100028276</t>
+          <t xml:space="preserve">100026096</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t xml:space="preserve">4</t>
+          <t xml:space="preserve">3</t>
         </is>
       </c>
       <c r="J32">
-        <v>146</v>
+        <v>241</v>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t xml:space="preserve">311734449</t>
+          <t xml:space="preserve">311736736</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
@@ -2399,7 +2399,7 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t xml:space="preserve">2034-01-22</t>
+          <t xml:space="preserve">2034-02-02</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
@@ -2441,7 +2441,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Godthåbsvej 21C</t>
+          <t xml:space="preserve">Gustav Johannsens Vej 21</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -2451,20 +2451,20 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t xml:space="preserve">100026096</t>
+          <t xml:space="preserve">100029332</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t xml:space="preserve">3</t>
+          <t xml:space="preserve">8</t>
         </is>
       </c>
       <c r="J33">
-        <v>241</v>
+        <v>86</v>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t xml:space="preserve">311736736</t>
+          <t xml:space="preserve">311736740</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
@@ -2516,7 +2516,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gustav Johannsens Vej 21</t>
+          <t xml:space="preserve">P.G. Ramms Alle 26</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2526,20 +2526,20 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t xml:space="preserve">100029332</t>
+          <t xml:space="preserve">100029627</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t xml:space="preserve">8</t>
+          <t xml:space="preserve">2</t>
         </is>
       </c>
       <c r="J34">
-        <v>86</v>
+        <v>110</v>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t xml:space="preserve">311736740</t>
+          <t xml:space="preserve">311737458</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
@@ -2549,7 +2549,7 @@
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t xml:space="preserve">2034-02-02</t>
+          <t xml:space="preserve">2034-02-06</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
@@ -2591,7 +2591,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t xml:space="preserve">P.G. Ramms Alle 26</t>
+          <t xml:space="preserve">Roskildevej 42A</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -2601,20 +2601,20 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t xml:space="preserve">100029627</t>
+          <t xml:space="preserve">100029157</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t xml:space="preserve">2</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="J35">
-        <v>110</v>
+        <v>165</v>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t xml:space="preserve">311737458</t>
+          <t xml:space="preserve">311737456</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
@@ -2666,7 +2666,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t xml:space="preserve">Roskildevej 42A</t>
+          <t xml:space="preserve">Stockflethsvej 2</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -2676,7 +2676,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t xml:space="preserve">100029157</t>
+          <t xml:space="preserve">100029710</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -2685,11 +2685,11 @@
         </is>
       </c>
       <c r="J36">
-        <v>165</v>
+        <v>60</v>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t xml:space="preserve">311737456</t>
+          <t xml:space="preserve">311737445</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
@@ -2726,12 +2726,12 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Direkte ejer</t>
+          <t xml:space="preserve">Medejer</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Frederiksberg Kommune</t>
+          <t xml:space="preserve">FREDERIKSBERG IDRÆTS-UNION</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -2741,7 +2741,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Stockflethsvej 2</t>
+          <t xml:space="preserve">Mariendalsvej 21C</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -2751,20 +2751,20 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t xml:space="preserve">100029710</t>
+          <t xml:space="preserve">100028066, 100195373</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">2</t>
         </is>
       </c>
       <c r="J37">
-        <v>60</v>
+        <v>178</v>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t xml:space="preserve">311737445</t>
+          <t xml:space="preserve">311743861</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
@@ -2774,7 +2774,7 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t xml:space="preserve">2034-02-06</t>
+          <t xml:space="preserve">2034-03-08</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
@@ -2801,12 +2801,12 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t xml:space="preserve">Medejer</t>
+          <t xml:space="preserve">Direkte ejer</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREDERIKSBERG IDRÆTS-UNION</t>
+          <t xml:space="preserve">Frederiksberg Kommune</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -2816,7 +2816,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mariendalsvej 21C</t>
+          <t xml:space="preserve">Segelckesvej 7</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -2826,7 +2826,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t xml:space="preserve">100028066, 100195373</t>
+          <t xml:space="preserve">100030239</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -2835,21 +2835,21 @@
         </is>
       </c>
       <c r="J38">
-        <v>178</v>
+        <v>197</v>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t xml:space="preserve">311743861</t>
+          <t xml:space="preserve">311930765</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t xml:space="preserve">OBH Ingeniørservice A/S</t>
+          <t xml:space="preserve">TÜV SÜD Domutech A/S</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t xml:space="preserve">2034-03-08</t>
+          <t xml:space="preserve">2036-10-08</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">

</xml_diff>